<commit_message>
Repoint sensitivity + black-box TEA analyses at the surviving waste_heat package
- delete dead lcow_full_global_map_waste_heat_lumped.py (imported the
  lcow_random_global_map_* module removed in 7dc283e)
- delete npv_heatmap_waste_heat_lumped.py, superseded by npv_heatmap_waste_heat.py
- rename npv_heatmap_cycle.py / tornado_plot_cycle.py -> *_waste_heat.py and drop
  their now single-valued --model flag
- tornado_plot_oat.py: drop the waste_heat_lumped model, collapse to solar-only and
  strip the figsize/fonts params no caller passes
- rewrite lcow_site_breakdown against the survivor's parameter_sweep API
- black_box_tea waste-heat workbook now imports waste_heat

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/black_box_tea/waste_heat/waste_heat_sawh_tea.xlsx
+++ b/analysis/black_box_tea/waste_heat/waste_heat_sawh_tea.xlsx
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>51.14969106729058</v>
+        <v>46.26848476541103</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>0.003850358875959504</v>
+        <v>0.003389982916127594</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>18.66963723956106</v>
+        <v>16.88799693937503</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>18.48294086716545</v>
+        <v>16.71911696998128</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1065,177 +1065,161 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Transfer pump (18)</t>
+          <t>Vacuum pump (28)</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>550</v>
+        <v>3500</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>550</v>
+        <v>3500</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>36.9686391782725</v>
+        <v>235.2549765890068</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Vacuum pump (28)</t>
+          <t>Chambers (22A, 22B) with door assemblies (38)</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>3500</v>
+        <v>1050</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>3500</v>
+        <v>1050</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>235.2549765890068</v>
+        <v>70.57649297670204</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Chambers (22A, 22B) with door assemblies (38)</t>
+          <t>Three-way valve (32) + check valve (30)</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>1050</v>
+        <v>275</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>1050</v>
+        <v>275</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>70.57649297670204</v>
+        <v>18.48431958913625</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Three-way valve (32) + check valve (30)</t>
+          <t>Condenser (24)</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>275</v>
+        <v>850</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>275</v>
+        <v>850</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>18.48431958913625</v>
+        <v>57.13335145733023</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Condenser (24)</t>
+          <t>Coolant source (26)</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>850</v>
+        <v>325</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>850</v>
+        <v>325</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>57.13335145733023</v>
+        <v>21.8451049689792</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Coolant source (26)</t>
+          <t>Water pump (34)</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>325</v>
+        <v>165</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>325</v>
+        <v>165</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>21.8451049689792</v>
+        <v>11.09059175348175</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Water pump (34)</t>
+          <t>Controller (16) + sensors (36)</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>165</v>
+        <v>800</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>165</v>
+        <v>800</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>11.09059175348175</v>
+        <v>53.77256607748727</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Controller (16) + sensors (36)</t>
+          <t>Purge pump (234)</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>53.77256607748727</v>
+        <v>26.88628303874363</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Purge pump (234)</t>
+          <t>Structural housing, manifolds, plumbing, fasteners</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>400</v>
+        <v>1350</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>400</v>
+        <v>1350</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>26.88628303874363</v>
+        <v>90.74120525575977</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Structural housing, manifolds, plumbing, fasteners</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>1350</v>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>90.74120525575977</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Total device CAPEX</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
-        <v>9265</v>
-      </c>
-      <c r="C14" s="10" t="n">
-        <v>9265</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>622.7535308848994</v>
+      <c r="B13" s="10" t="n">
+        <v>8715</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>8715</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>585.7848917066269</v>
       </c>
     </row>
   </sheetData>
@@ -1249,7 +1233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1321,170 +1305,140 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Transfer pump (18)</t>
+          <t>Vacuum pump (28)</t>
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>19.6133</v>
+        <v>45</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0.55</v>
+        <v>0.35</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>35.66054545454545</v>
+        <v>128.5714285714286</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>312.3863781818181</v>
+        <v>563.1428571428572</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>31.23863781818181</v>
+        <v>56.31428571428572</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>HTF loop: ρgHQ at ṁ=0.25 kg/s/m², H=8 m</t>
+          <t>Roughing pump during desorption half-cycles</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Vacuum pump (28)</t>
+          <t>Water pump (34)</t>
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>128.5714285714286</v>
+        <v>6</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>563.1428571428572</v>
+        <v>4.38</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>56.31428571428572</v>
+        <v>0.438</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Roughing pump during desorption half-cycles</t>
+          <t>Product-water transfer</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Water pump (34)</t>
+          <t>Purge pump (234)</t>
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>6</v>
+        <v>17.77777777777778</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>4.38</v>
+        <v>6.48888888888889</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.438</v>
+        <v>0.6488888888888891</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Product-water transfer</t>
+          <t>Manifold / valve purge</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Purge pump (234)</t>
+          <t>Controller (16) + sensors (36)</t>
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.45</v>
+        <v>0.85</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>17.77777777777778</v>
+        <v>2.941176470588236</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>6.48888888888889</v>
+        <v>25.76470588235295</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>0.6488888888888891</v>
+        <v>2.576470588235295</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Manifold / valve purge</t>
+          <t>Controls and instrumentation</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Controller (16) + sensors (36)</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>24</v>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>2.941176470588236</v>
-      </c>
-      <c r="F9" s="8" t="n">
-        <v>25.76470588235295</v>
-      </c>
-      <c r="G9" s="8" t="n">
-        <v>2.576470588235295</v>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Controls and instrumentation</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Total parasitic electricity</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="10" t="n">
-        <v>912.1628300959171</v>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>91.21628300959172</v>
-      </c>
-      <c r="H10" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="10" t="n">
+        <v>599.7764519140991</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>59.97764519140991</v>
+      </c>
+      <c r="H9" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1500,7 +1454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1550,7 +1504,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>463.25</v>
+        <v>435.75</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -1617,7 +1571,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Transfer pump (18)</t>
+          <t>Electricity: Vacuum pump (28)</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
@@ -1626,7 +1580,7 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>31.23863781818181</v>
+        <v>56.31428571428572</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
@@ -1637,7 +1591,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Vacuum pump (28)</t>
+          <t>Electricity: Water pump (34)</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
@@ -1646,7 +1600,7 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>56.31428571428572</v>
+        <v>0.438</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
@@ -1657,7 +1611,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Water pump (34)</t>
+          <t>Electricity: Purge pump (234)</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
@@ -1666,7 +1620,7 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>0.438</v>
+        <v>0.6488888888888891</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
@@ -1677,7 +1631,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Purge pump (234)</t>
+          <t>Electricity: Controller (16) + sensors (36)</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
@@ -1686,7 +1640,7 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>0.6488888888888891</v>
+        <v>2.576470588235295</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -1697,7 +1651,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Controller (16) + sensors (36)</t>
+          <t>Extra cycling energy</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
@@ -1706,75 +1660,55 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>2.576470588235295</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Shaft power / motor efficiency × hours</t>
+          <t>Energy above one half-cycle per day</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Extra cycling energy</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Energy above one half-cycle per day</t>
-        </is>
-      </c>
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Subtotal — fixed OPEX</t>
+        </is>
+      </c>
       <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
+      <c r="C14" s="8" t="n">
+        <v>440.6807500566884</v>
+      </c>
       <c r="D14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Subtotal — fixed OPEX</t>
+          <t>Subtotal — variable OPEX</t>
         </is>
       </c>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="8" t="n">
-        <v>468.1807500566884</v>
+        <v>59.97764519140991</v>
       </c>
       <c r="D15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Subtotal — variable OPEX</t>
+          <t>Total OPEX</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
-      <c r="C16" s="8" t="n">
-        <v>91.21628300959172</v>
+      <c r="C16" s="10" t="n">
+        <v>500.6583952480983</v>
       </c>
       <c r="D16" s="3" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Total OPEX</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="10" t="n">
-        <v>559.3970330662801</v>
-      </c>
-      <c r="D17" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1787,7 +1721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1833,7 +1767,7 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>622.7535308848994</v>
+        <v>585.7848917066269</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
@@ -1848,7 +1782,7 @@
         </is>
       </c>
       <c r="B6" s="14" t="n">
-        <v>468.1807500566884</v>
+        <v>440.6807500566884</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -1863,7 +1797,7 @@
         </is>
       </c>
       <c r="B7" s="14" t="n">
-        <v>91.21628300959172</v>
+        <v>59.97764519140991</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -1878,7 +1812,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>1182.150563951179</v>
+        <v>1086.443286954725</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -1893,7 +1827,7 @@
         </is>
       </c>
       <c r="B9" s="14" t="n">
-        <v>18.66963723956106</v>
+        <v>16.88799693937503</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -1908,7 +1842,7 @@
         </is>
       </c>
       <c r="B10" s="14" t="n">
-        <v>18.48294086716545</v>
+        <v>16.71911696998128</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -1928,7 +1862,7 @@
         </is>
       </c>
       <c r="B12" s="16" t="n">
-        <v>63.9590080630104</v>
+        <v>64.9820973742456</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
@@ -1975,189 +1909,189 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Transfer pump (18)</t>
+          <t>CAPEX: Vacuum pump (28)</t>
         </is>
       </c>
       <c r="B17" s="14" t="n">
-        <v>36.9686391782725</v>
+        <v>235.2549765890068</v>
       </c>
       <c r="C17" s="14" t="n">
-        <v>2.000149188592952</v>
+        <v>14.07101684923916</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Vacuum pump (28)</t>
+          <t>CAPEX: Chambers (22A, 22B) with door assemblies (38)</t>
         </is>
       </c>
       <c r="B18" s="14" t="n">
-        <v>235.2549765890068</v>
+        <v>70.57649297670204</v>
       </c>
       <c r="C18" s="14" t="n">
-        <v>12.72822210922788</v>
+        <v>4.221305054771746</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Chambers (22A, 22B) with door assemblies (38)</t>
+          <t>CAPEX: Three-way valve (32) + check valve (30)</t>
         </is>
       </c>
       <c r="B19" s="14" t="n">
-        <v>70.57649297670204</v>
+        <v>18.48431958913625</v>
       </c>
       <c r="C19" s="14" t="n">
-        <v>3.818466632768364</v>
+        <v>1.105579895297362</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Three-way valve (32) + check valve (30)</t>
+          <t>CAPEX: Condenser (24)</t>
         </is>
       </c>
       <c r="B20" s="14" t="n">
-        <v>18.48431958913625</v>
+        <v>57.13335145733023</v>
       </c>
       <c r="C20" s="14" t="n">
-        <v>1.000074594296476</v>
+        <v>3.417246949100938</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Condenser (24)</t>
+          <t>CAPEX: Coolant source (26)</t>
         </is>
       </c>
       <c r="B21" s="14" t="n">
-        <v>57.13335145733023</v>
+        <v>21.8451049689792</v>
       </c>
       <c r="C21" s="14" t="n">
-        <v>3.0911396550982</v>
+        <v>1.306594421715064</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Coolant source (26)</t>
+          <t>CAPEX: Water pump (34)</t>
         </is>
       </c>
       <c r="B22" s="14" t="n">
-        <v>21.8451049689792</v>
+        <v>11.09059175348175</v>
       </c>
       <c r="C22" s="14" t="n">
-        <v>1.181906338714017</v>
+        <v>0.6633479371784173</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Water pump (34)</t>
+          <t>CAPEX: Controller (16) + sensors (36)</t>
         </is>
       </c>
       <c r="B23" s="14" t="n">
-        <v>11.09059175348175</v>
+        <v>53.77256607748727</v>
       </c>
       <c r="C23" s="14" t="n">
-        <v>0.6000447565778858</v>
+        <v>3.216232422683235</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Controller (16) + sensors (36)</t>
+          <t>CAPEX: Purge pump (234)</t>
         </is>
       </c>
       <c r="B24" s="14" t="n">
-        <v>53.77256607748727</v>
+        <v>26.88628303874363</v>
       </c>
       <c r="C24" s="14" t="n">
-        <v>2.909307910680658</v>
+        <v>1.608116211341618</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Purge pump (234)</t>
+          <t>CAPEX: Structural housing, manifolds, plumbing, fasteners</t>
         </is>
       </c>
       <c r="B25" s="14" t="n">
-        <v>26.88628303874363</v>
+        <v>90.74120525575977</v>
       </c>
       <c r="C25" s="14" t="n">
-        <v>1.454653955340329</v>
+        <v>5.427392213277959</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>CAPEX: Structural housing, manifolds, plumbing, fasteners</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B26" s="14" t="n">
-        <v>90.74120525575977</v>
+        <v>435.75</v>
       </c>
       <c r="C26" s="14" t="n">
-        <v>4.90945709927361</v>
+        <v>26.06297932973239</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Hydrogel: salt</t>
         </is>
       </c>
       <c r="B27" s="14" t="n">
-        <v>463.25</v>
+        <v>4.427727452860338</v>
       </c>
       <c r="C27" s="14" t="n">
-        <v>25.06365211733993</v>
+        <v>0.2648302216444925</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Hydrogel: salt</t>
+          <t>Hydrogel: acrylamide</t>
         </is>
       </c>
       <c r="B28" s="14" t="n">
-        <v>4.427727452860338</v>
+        <v>0.4870500198146372</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>0.2395575187239873</v>
+        <v>0.02913132438089418</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Hydrogel: acrylamide</t>
+          <t>Hydrogel: additives</t>
         </is>
       </c>
       <c r="B29" s="14" t="n">
-        <v>0.4870500198146372</v>
+        <v>0.01597258401344838</v>
       </c>
       <c r="C29" s="14" t="n">
-        <v>0.02635132705963861</v>
+        <v>0.0009553485415603424</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Hydrogel: additives</t>
+          <t>Fixed energy</t>
         </is>
       </c>
       <c r="B30" s="14" t="n">
-        <v>0.01597258401344838</v>
+        <v>0</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>0.0008641797930449119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Fixed energy</t>
+          <t>Electricity (supplemental heat)</t>
         </is>
       </c>
       <c r="B31" s="14" t="n">
@@ -2170,103 +2104,77 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Electricity (supplemental heat)</t>
+          <t>Electricity: Vacuum pump (28)</t>
         </is>
       </c>
       <c r="B32" s="14" t="n">
-        <v>0</v>
+        <v>56.31428571428572</v>
       </c>
       <c r="C32" s="14" t="n">
-        <v>0</v>
+        <v>3.368257176225067</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Transfer pump (18)</t>
+          <t>Electricity: Water pump (34)</t>
         </is>
       </c>
       <c r="B33" s="14" t="n">
-        <v>31.23863781818181</v>
+        <v>0.438</v>
       </c>
       <c r="C33" s="14" t="n">
-        <v>1.690133515152699</v>
+        <v>0.02619755581508385</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Vacuum pump (28)</t>
+          <t>Electricity: Purge pump (234)</t>
         </is>
       </c>
       <c r="B34" s="14" t="n">
-        <v>56.31428571428572</v>
+        <v>0.6488888888888891</v>
       </c>
       <c r="C34" s="14" t="n">
-        <v>3.046824967899283</v>
+        <v>0.03881119380012423</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Water pump (34)</t>
+          <t>Electricity: Controller (16) + sensors (36)</t>
         </is>
       </c>
       <c r="B35" s="14" t="n">
-        <v>0.438</v>
+        <v>2.576470588235295</v>
       </c>
       <c r="C35" s="14" t="n">
-        <v>0.02369752752810553</v>
+        <v>0.1541032695004932</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Electricity: Purge pump (234)</t>
+          <t>Extra cycling energy</t>
         </is>
       </c>
       <c r="B36" s="14" t="n">
-        <v>0.6488888888888891</v>
+        <v>0</v>
       </c>
       <c r="C36" s="14" t="n">
-        <v>0.03510744818978598</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Electricity: Controller (16) + sensors (36)</t>
-        </is>
-      </c>
-      <c r="B37" s="14" t="n">
-        <v>2.576470588235295</v>
-      </c>
-      <c r="C37" s="14" t="n">
-        <v>0.139397220753562</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>Extra cycling energy</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C38" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>Total (check)</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n"/>
-      <c r="C39" s="17" t="n">
-        <v>63.95900806301041</v>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="17" t="n">
+        <v>64.9820973742456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>